<commit_message>
Update PCB mounting hardware footprints
</commit_message>
<xml_diff>
--- a/outputs/bom_aggregate/BOM_集計.xlsx
+++ b/outputs/bom_aggregate/BOM_集計.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fd25e66c625c5f55/ドキュメント/Bifrost/outputs/bom_aggregate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="106" documentId="11_A1BEE109FB28F8718521FC0C9678AB06B2C69440" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F22F7DD5-B03B-4F8F-B259-F437E1A239A5}"/>
+  <xr:revisionPtr revIDLastSave="113" documentId="11_A1BEE109FB28F8718521FC0C9678AB06B2C69440" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4C56430-AF26-49ED-A950-2E557D28A264}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -875,7 +875,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -903,12 +903,6 @@
     <xf numFmtId="3" fontId="6" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -924,7 +918,28 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -942,6 +957,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2432,32 +2451,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
     </row>
     <row r="2" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
     </row>
     <row r="4" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
@@ -2494,44 +2513,43 @@
         <v>184</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A5" s="11" t="s">
+    <row r="5" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="20" t="s">
         <v>200</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="D5" s="6">
-        <v>2</v>
-      </c>
-      <c r="E5" s="6">
-        <v>1</v>
-      </c>
-      <c r="F5" s="6">
-        <v>0</v>
-      </c>
-      <c r="G5" s="6">
-        <v>0</v>
-      </c>
-      <c r="H5" s="6">
-        <v>0</v>
-      </c>
-      <c r="I5" s="8">
+      <c r="D5" s="17">
+        <v>2</v>
+      </c>
+      <c r="E5" s="17">
+        <v>1</v>
+      </c>
+      <c r="F5" s="17">
+        <v>0</v>
+      </c>
+      <c r="G5" s="17">
+        <v>0</v>
+      </c>
+      <c r="H5" s="17">
+        <v>0</v>
+      </c>
+      <c r="I5" s="18">
         <v>3</v>
       </c>
-      <c r="J5" s="16" t="s">
+      <c r="J5" s="21" t="s">
         <v>201</v>
       </c>
-      <c r="K5" s="14"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="9" t="s">
         <v>177</v>
       </c>
       <c r="C6" s="5" t="s">
@@ -2559,12 +2577,12 @@
       <c r="J6" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="K6" s="12">
+      <c r="K6" s="10">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="9" t="s">
         <v>179</v>
       </c>
       <c r="B7" s="5" t="s">
@@ -2593,12 +2611,12 @@
       <c r="J7" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="K7" s="12">
+      <c r="K7" s="10">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="9" t="s">
         <v>180</v>
       </c>
       <c r="B8" s="5" t="s">
@@ -2629,12 +2647,12 @@
       <c r="J8" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="K8" s="12">
+      <c r="K8" s="10">
         <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="9" t="s">
         <v>210</v>
       </c>
       <c r="B9" s="5" t="s">
@@ -2665,12 +2683,12 @@
       <c r="J9" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="K9" s="12">
+      <c r="K9" s="10">
         <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="9" t="s">
         <v>181</v>
       </c>
       <c r="B10" s="5" t="s">
@@ -2701,48 +2719,48 @@
       <c r="J10" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="K10" s="12">
+      <c r="K10" s="10">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="37.5" x14ac:dyDescent="0.4">
-      <c r="A11" s="11" t="s">
+    <row r="11" spans="1:11" s="12" customFormat="1" ht="37.5" x14ac:dyDescent="0.4">
+      <c r="A11" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="D11" s="6">
-        <v>2</v>
-      </c>
-      <c r="E11" s="6">
-        <v>2</v>
-      </c>
-      <c r="F11" s="6">
-        <v>2</v>
-      </c>
-      <c r="G11" s="6">
+      <c r="D11" s="17">
+        <v>2</v>
+      </c>
+      <c r="E11" s="17">
+        <v>2</v>
+      </c>
+      <c r="F11" s="17">
+        <v>2</v>
+      </c>
+      <c r="G11" s="17">
         <v>3</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="17">
         <v>3</v>
       </c>
-      <c r="I11" s="8">
+      <c r="I11" s="18">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="J11" s="7" t="s">
+      <c r="J11" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="K11" s="15" t="s">
+      <c r="K11" s="13" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="9" t="s">
         <v>209</v>
       </c>
       <c r="B12" s="5" t="s">
@@ -2773,12 +2791,12 @@
       <c r="J12" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="K12" s="12">
+      <c r="K12" s="10">
         <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="9" t="s">
         <v>208</v>
       </c>
       <c r="B13" s="5" t="s">
@@ -2809,12 +2827,12 @@
       <c r="J13" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="K13" s="12">
+      <c r="K13" s="10">
         <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="9" t="s">
         <v>211</v>
       </c>
       <c r="B14" s="5" t="s">
@@ -2845,48 +2863,48 @@
       <c r="J14" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="K14" s="12">
+      <c r="K14" s="10">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A15" s="5" t="s">
+    <row r="15" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="D15" s="6">
-        <v>1</v>
-      </c>
-      <c r="E15" s="6">
-        <v>1</v>
-      </c>
-      <c r="F15" s="6">
-        <v>0</v>
-      </c>
-      <c r="G15" s="6">
-        <v>0</v>
-      </c>
-      <c r="H15" s="6">
-        <v>0</v>
-      </c>
-      <c r="I15" s="8">
+      <c r="D15" s="17">
+        <v>1</v>
+      </c>
+      <c r="E15" s="17">
+        <v>1</v>
+      </c>
+      <c r="F15" s="17">
+        <v>0</v>
+      </c>
+      <c r="G15" s="17">
+        <v>0</v>
+      </c>
+      <c r="H15" s="17">
+        <v>0</v>
+      </c>
+      <c r="I15" s="18">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="J15" s="7" t="s">
+      <c r="J15" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="K15" s="15" t="s">
+      <c r="K15" s="13" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="9" t="s">
         <v>182</v>
       </c>
       <c r="B16" s="5" t="s">
@@ -2917,12 +2935,12 @@
       <c r="J16" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="K16" s="12">
+      <c r="K16" s="10">
         <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="9" t="s">
         <v>207</v>
       </c>
       <c r="B17" s="5" t="s">
@@ -2953,12 +2971,12 @@
       <c r="J17" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="K17" s="12">
+      <c r="K17" s="10">
         <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="9" t="s">
         <v>206</v>
       </c>
       <c r="B18" s="5" t="s">
@@ -2989,46 +3007,45 @@
       <c r="J18" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="K18" s="12">
+      <c r="K18" s="10">
         <v>100</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A19" s="5" t="s">
+    <row r="19" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="D19" s="6">
-        <v>2</v>
-      </c>
-      <c r="E19" s="6">
-        <v>2</v>
-      </c>
-      <c r="F19" s="6">
-        <v>0</v>
-      </c>
-      <c r="G19" s="6">
-        <v>0</v>
-      </c>
-      <c r="H19" s="6">
-        <v>0</v>
-      </c>
-      <c r="I19" s="8">
+      <c r="D19" s="17">
+        <v>2</v>
+      </c>
+      <c r="E19" s="17">
+        <v>2</v>
+      </c>
+      <c r="F19" s="17">
+        <v>0</v>
+      </c>
+      <c r="G19" s="17">
+        <v>0</v>
+      </c>
+      <c r="H19" s="17">
+        <v>0</v>
+      </c>
+      <c r="I19" s="18">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="J19" s="7" t="s">
+      <c r="J19" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="K19" s="14"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="9" t="s">
         <v>205</v>
       </c>
       <c r="B20" s="5" t="s">
@@ -3059,46 +3076,45 @@
       <c r="J20" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="K20" s="12">
+      <c r="K20" s="10">
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A21" s="5" t="s">
+    <row r="21" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="D21" s="6">
-        <v>2</v>
-      </c>
-      <c r="E21" s="6">
-        <v>2</v>
-      </c>
-      <c r="F21" s="6">
-        <v>0</v>
-      </c>
-      <c r="G21" s="6">
-        <v>0</v>
-      </c>
-      <c r="H21" s="6">
-        <v>1</v>
-      </c>
-      <c r="I21" s="8">
+      <c r="D21" s="17">
+        <v>2</v>
+      </c>
+      <c r="E21" s="17">
+        <v>2</v>
+      </c>
+      <c r="F21" s="17">
+        <v>0</v>
+      </c>
+      <c r="G21" s="17">
+        <v>0</v>
+      </c>
+      <c r="H21" s="17">
+        <v>1</v>
+      </c>
+      <c r="I21" s="18">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="J21" s="7" t="s">
+      <c r="J21" s="19" t="s">
         <v>156</v>
       </c>
-      <c r="K21" s="14"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="9" t="s">
         <v>204</v>
       </c>
       <c r="B22" s="5" t="s">
@@ -3129,12 +3145,12 @@
       <c r="J22" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="K22" s="12">
+      <c r="K22" s="10">
         <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="9" t="s">
         <v>203</v>
       </c>
       <c r="B23" s="5" t="s">
@@ -3165,12 +3181,12 @@
       <c r="J23" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="K23" s="12">
+      <c r="K23" s="10">
         <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="9" t="s">
         <v>202</v>
       </c>
       <c r="B24" s="5" t="s">
@@ -3201,12 +3217,12 @@
       <c r="J24" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="K24" s="12">
+      <c r="K24" s="10">
         <v>100</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="9" t="s">
         <v>183</v>
       </c>
       <c r="B25" s="5" t="s">
@@ -3235,48 +3251,48 @@
       <c r="J25" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="K25" s="12">
+      <c r="K25" s="10">
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A26" s="11" t="s">
+    <row r="26" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="20" t="s">
         <v>185</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="D26" s="6">
-        <v>1</v>
-      </c>
-      <c r="E26" s="6">
-        <v>1</v>
-      </c>
-      <c r="F26" s="6">
-        <v>0</v>
-      </c>
-      <c r="G26" s="6">
-        <v>0</v>
-      </c>
-      <c r="H26" s="6">
-        <v>0</v>
-      </c>
-      <c r="I26" s="8">
+      <c r="D26" s="17">
+        <v>1</v>
+      </c>
+      <c r="E26" s="17">
+        <v>1</v>
+      </c>
+      <c r="F26" s="17">
+        <v>0</v>
+      </c>
+      <c r="G26" s="17">
+        <v>0</v>
+      </c>
+      <c r="H26" s="17">
+        <v>0</v>
+      </c>
+      <c r="I26" s="18">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="J26" s="7" t="s">
+      <c r="J26" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="K26" s="14">
+      <c r="K26" s="12">
         <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="9" t="s">
         <v>186</v>
       </c>
       <c r="B27" s="5" t="s">
@@ -3307,12 +3323,12 @@
       <c r="J27" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="K27" s="12">
+      <c r="K27" s="10">
         <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A28" s="11" t="s">
+      <c r="A28" s="9" t="s">
         <v>187</v>
       </c>
       <c r="B28" s="5" t="s">
@@ -3343,12 +3359,12 @@
       <c r="J28" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="K28" s="12">
+      <c r="K28" s="10">
         <v>20</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A29" s="11" t="s">
+      <c r="A29" s="9" t="s">
         <v>188</v>
       </c>
       <c r="B29" s="5" t="s">
@@ -3379,7 +3395,7 @@
       <c r="J29" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="K29" s="12">
+      <c r="K29" s="10">
         <v>10</v>
       </c>
     </row>
@@ -3415,47 +3431,46 @@
       <c r="J30" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="K30" s="13"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A31" s="5" t="s">
+      <c r="K30" s="11"/>
+    </row>
+    <row r="31" spans="1:11" s="12" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A31" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C31" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="D31" s="6">
-        <v>0</v>
-      </c>
-      <c r="E31" s="6">
-        <v>0</v>
-      </c>
-      <c r="F31" s="6">
-        <v>0</v>
-      </c>
-      <c r="G31" s="6">
-        <v>0</v>
-      </c>
-      <c r="H31" s="6">
-        <v>1</v>
-      </c>
-      <c r="I31" s="8">
+      <c r="D31" s="17">
+        <v>0</v>
+      </c>
+      <c r="E31" s="17">
+        <v>0</v>
+      </c>
+      <c r="F31" s="17">
+        <v>0</v>
+      </c>
+      <c r="G31" s="17">
+        <v>0</v>
+      </c>
+      <c r="H31" s="17">
+        <v>1</v>
+      </c>
+      <c r="I31" s="18">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="J31" s="7" t="s">
+      <c r="J31" s="19" t="s">
         <v>166</v>
       </c>
-      <c r="K31" s="14"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A32" s="11" t="s">
+      <c r="A32" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="9" t="s">
         <v>189</v>
       </c>
       <c r="C32" s="5" t="s">
@@ -3483,12 +3498,12 @@
       <c r="J32" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="K32" s="12">
+      <c r="K32" s="10">
         <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A33" s="11" t="s">
+      <c r="A33" s="9" t="s">
         <v>191</v>
       </c>
       <c r="B33" s="5" t="s">
@@ -3519,12 +3534,12 @@
       <c r="J33" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="K33" s="12">
+      <c r="K33" s="10">
         <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A34" s="11" t="s">
+      <c r="A34" s="9" t="s">
         <v>192</v>
       </c>
       <c r="B34" s="5" t="s">
@@ -3555,12 +3570,12 @@
       <c r="J34" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="K34" s="12">
+      <c r="K34" s="10">
         <v>50</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A35" s="11" t="s">
+      <c r="A35" s="9" t="s">
         <v>193</v>
       </c>
       <c r="B35" s="5" t="s">
@@ -3591,12 +3606,12 @@
       <c r="J35" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="K35" s="12">
+      <c r="K35" s="10">
         <v>5</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A36" s="11" t="s">
+      <c r="A36" s="9" t="s">
         <v>194</v>
       </c>
       <c r="B36" s="5" t="s">
@@ -3627,12 +3642,12 @@
       <c r="J36" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="K36" s="12">
+      <c r="K36" s="10">
         <v>10</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A37" s="11" t="s">
+      <c r="A37" s="9" t="s">
         <v>195</v>
       </c>
       <c r="B37" s="5" t="s">
@@ -3663,7 +3678,7 @@
       <c r="J37" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="K37" s="12">
+      <c r="K37" s="10">
         <v>20</v>
       </c>
     </row>

</xml_diff>